<commit_message>
minor fixes and code updates
</commit_message>
<xml_diff>
--- a/Data/Rules/Bradley Caldwell Rules Matrix.xlsx
+++ b/Data/Rules/Bradley Caldwell Rules Matrix.xlsx
@@ -1042,10 +1042,10 @@
         <v>0</v>
       </c>
       <c r="AJ2">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="AK2">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="AL2" t="b">
         <v>1</v>
@@ -1164,10 +1164,10 @@
         <v>0</v>
       </c>
       <c r="AJ3">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="AK3">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="AL3" t="b">
         <v>1</v>
@@ -1196,10 +1196,10 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="G4">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="H4" t="b">
         <v>0</v>
@@ -1214,82 +1214,82 @@
         <v>0</v>
       </c>
       <c r="L4">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="M4">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="N4" t="b">
         <v>0</v>
       </c>
       <c r="O4">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="P4">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="Q4" t="b">
         <v>0</v>
       </c>
       <c r="R4">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="S4">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="T4" t="b">
         <v>0</v>
       </c>
       <c r="U4">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="V4">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="W4" t="b">
         <v>0</v>
       </c>
       <c r="X4">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="Y4">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="Z4" t="b">
         <v>0</v>
       </c>
       <c r="AA4">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="AB4">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="AC4" t="b">
         <v>0</v>
       </c>
       <c r="AD4">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="AE4">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="AF4" t="b">
         <v>0</v>
       </c>
       <c r="AG4">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="AH4">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="AI4" t="b">
         <v>0</v>
       </c>
       <c r="AJ4">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="AK4">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="AL4" t="b">
         <v>1</v>
@@ -1318,10 +1318,10 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="G5">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="H5" t="b">
         <v>0</v>
@@ -1336,82 +1336,82 @@
         <v>0</v>
       </c>
       <c r="L5">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="M5">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="N5" t="b">
         <v>0</v>
       </c>
       <c r="O5">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="P5">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="Q5" t="b">
         <v>0</v>
       </c>
       <c r="R5">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="S5">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="T5" t="b">
         <v>0</v>
       </c>
       <c r="U5">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="V5">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="W5" t="b">
         <v>0</v>
       </c>
       <c r="X5">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="Y5">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="Z5" t="b">
         <v>0</v>
       </c>
       <c r="AA5">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="AB5">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="AC5" t="b">
         <v>0</v>
       </c>
       <c r="AD5">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="AE5">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="AF5" t="b">
         <v>0</v>
       </c>
       <c r="AG5">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="AH5">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="AI5" t="b">
         <v>0</v>
       </c>
       <c r="AJ5">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="AK5">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="AL5" t="b">
         <v>1</v>
@@ -1533,7 +1533,7 @@
         <v>25</v>
       </c>
       <c r="AK6">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="AL6" t="b">
         <v>1</v>
@@ -1652,10 +1652,10 @@
         <v>0</v>
       </c>
       <c r="AJ7">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="AK7">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="AL7" t="b">
         <v>1</v>
@@ -1684,10 +1684,10 @@
         <v>0</v>
       </c>
       <c r="F8">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="G8">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="H8" t="b">
         <v>0</v>
@@ -1702,82 +1702,82 @@
         <v>0</v>
       </c>
       <c r="L8">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="M8">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="N8" t="b">
         <v>0</v>
       </c>
       <c r="O8">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="P8">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="Q8" t="b">
         <v>0</v>
       </c>
       <c r="R8">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="S8">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="T8" t="b">
         <v>0</v>
       </c>
       <c r="U8">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="V8">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="W8" t="b">
         <v>0</v>
       </c>
       <c r="X8">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="Y8">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="Z8" t="b">
         <v>0</v>
       </c>
       <c r="AA8">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="AB8">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="AC8" t="b">
         <v>0</v>
       </c>
       <c r="AD8">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="AE8">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="AF8" t="b">
         <v>0</v>
       </c>
       <c r="AG8">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="AH8">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="AI8" t="b">
         <v>0</v>
       </c>
       <c r="AJ8">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="AK8">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="AL8" t="b">
         <v>1</v>
@@ -1800,43 +1800,43 @@
         <v>148</v>
       </c>
       <c r="D9">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
       </c>
       <c r="F9">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="G9">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="H9" t="b">
         <v>0</v>
       </c>
       <c r="I9">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="J9">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="K9" t="b">
         <v>0</v>
       </c>
       <c r="L9">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="M9">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="N9" t="b">
         <v>0</v>
       </c>
       <c r="O9">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="P9">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="Q9" t="b">
         <v>0</v>
@@ -1851,16 +1851,16 @@
         <v>0</v>
       </c>
       <c r="U9">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="V9">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="W9" t="b">
         <v>0</v>
       </c>
       <c r="X9">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="Y9">
         <v>25</v>
@@ -1869,16 +1869,16 @@
         <v>0</v>
       </c>
       <c r="AA9">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="AB9">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="AC9" t="b">
         <v>0</v>
       </c>
       <c r="AD9">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AE9">
         <v>25</v>
@@ -1887,19 +1887,19 @@
         <v>0</v>
       </c>
       <c r="AG9">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="AH9">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="AI9" t="b">
         <v>0</v>
       </c>
       <c r="AJ9">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="AK9">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="AL9" t="b">
         <v>1</v>
@@ -1964,10 +1964,10 @@
         <v>0</v>
       </c>
       <c r="R10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S10">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T10" t="b">
         <v>0</v>
@@ -1982,10 +1982,10 @@
         <v>0</v>
       </c>
       <c r="X10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Y10">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Z10" t="b">
         <v>0</v>
@@ -2000,10 +2000,10 @@
         <v>0</v>
       </c>
       <c r="AD10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AE10">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AF10" t="b">
         <v>0</v>
@@ -3794,10 +3794,10 @@
         <v>0</v>
       </c>
       <c r="R25">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S25">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="T25" t="b">
         <v>0</v>
@@ -3830,10 +3830,10 @@
         <v>0</v>
       </c>
       <c r="AD25">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AE25">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AF25" t="b">
         <v>0</v>
@@ -3916,10 +3916,10 @@
         <v>0</v>
       </c>
       <c r="R26">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S26">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="T26" t="b">
         <v>0</v>
@@ -3952,10 +3952,10 @@
         <v>0</v>
       </c>
       <c r="AD26">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AE26">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AF26" t="b">
         <v>0</v>
@@ -4038,10 +4038,10 @@
         <v>0</v>
       </c>
       <c r="R27">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S27">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="T27" t="b">
         <v>0</v>
@@ -4074,10 +4074,10 @@
         <v>0</v>
       </c>
       <c r="AD27">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AE27">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AF27" t="b">
         <v>0</v>
@@ -4160,10 +4160,10 @@
         <v>0</v>
       </c>
       <c r="R28">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S28">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="T28" t="b">
         <v>0</v>
@@ -4196,10 +4196,10 @@
         <v>0</v>
       </c>
       <c r="AD28">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AE28">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AF28" t="b">
         <v>0</v>
@@ -4404,10 +4404,10 @@
         <v>0</v>
       </c>
       <c r="R30">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S30">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="T30" t="b">
         <v>0</v>
@@ -4422,10 +4422,10 @@
         <v>0</v>
       </c>
       <c r="X30">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Y30">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Z30" t="b">
         <v>0</v>
@@ -4526,10 +4526,10 @@
         <v>0</v>
       </c>
       <c r="R31">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S31">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="T31" t="b">
         <v>0</v>
@@ -4544,10 +4544,10 @@
         <v>0</v>
       </c>
       <c r="X31">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Y31">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Z31" t="b">
         <v>0</v>
@@ -4648,10 +4648,10 @@
         <v>0</v>
       </c>
       <c r="R32">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S32">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="T32" t="b">
         <v>0</v>
@@ -4666,10 +4666,10 @@
         <v>0</v>
       </c>
       <c r="X32">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Y32">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Z32" t="b">
         <v>0</v>
@@ -5844,7 +5844,7 @@
         <v>1</v>
       </c>
       <c r="J42">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K42" t="b">
         <v>0</v>
@@ -5966,7 +5966,7 @@
         <v>1</v>
       </c>
       <c r="J43">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K43" t="b">
         <v>0</v>
@@ -6808,7 +6808,7 @@
         <v>0</v>
       </c>
       <c r="F50">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G50">
         <v>12</v>
@@ -6817,7 +6817,7 @@
         <v>0</v>
       </c>
       <c r="I50">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J50">
         <v>12</v>
@@ -6826,7 +6826,7 @@
         <v>0</v>
       </c>
       <c r="L50">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M50">
         <v>12</v>
@@ -6835,7 +6835,7 @@
         <v>0</v>
       </c>
       <c r="O50">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="P50">
         <v>12</v>
@@ -6844,7 +6844,7 @@
         <v>0</v>
       </c>
       <c r="R50">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="S50">
         <v>12</v>
@@ -6853,7 +6853,7 @@
         <v>0</v>
       </c>
       <c r="U50">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="V50">
         <v>12</v>
@@ -6862,7 +6862,7 @@
         <v>0</v>
       </c>
       <c r="X50">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="Y50">
         <v>12</v>
@@ -6871,7 +6871,7 @@
         <v>0</v>
       </c>
       <c r="AA50">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AB50">
         <v>12</v>
@@ -6889,7 +6889,7 @@
         <v>0</v>
       </c>
       <c r="AG50">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AH50">
         <v>12</v>
@@ -6898,7 +6898,7 @@
         <v>0</v>
       </c>
       <c r="AJ50">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AK50">
         <v>12</v>

</xml_diff>